<commit_message>
feat: apply procurement prices from EVN Vinh Tan 4 package IB2600096765 (divided by 1.08 for pre-VAT)
</commit_message>
<xml_diff>
--- a/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_2026_10_SHEET.xlsx
+++ b/backend/data/DU_TOAN_QUAN_TRAC_MOI_TRUONG_2026_10_SHEET.xlsx
@@ -47624,7 +47624,7 @@
         <v>185250</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>191100</v>
+        <v>370000</v>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2">
@@ -47667,7 +47667,7 @@
         <v>228</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>235</v>
+        <v>370</v>
       </c>
       <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3">
@@ -47839,7 +47839,7 @@
         <v>1140</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>1180</v>
+        <v>59100</v>
       </c>
       <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3">
@@ -48742,7 +48742,7 @@
         <v>185250</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>191100</v>
+        <v>40000</v>
       </c>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2">
@@ -48785,7 +48785,7 @@
         <v>185250</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>191100</v>
+        <v>40000</v>
       </c>
       <c r="K36" s="3" t="inlineStr"/>
       <c r="L36" s="3">
@@ -48828,7 +48828,7 @@
         <v>228</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>235</v>
+        <v>40</v>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2">
@@ -48871,7 +48871,7 @@
         <v>228</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>235</v>
+        <v>40</v>
       </c>
       <c r="K38" s="3" t="inlineStr"/>
       <c r="L38" s="3">
@@ -48957,7 +48957,7 @@
         <v>8080</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>8330</v>
+        <v>4780</v>
       </c>
       <c r="K40" s="3" t="inlineStr"/>
       <c r="L40" s="3">
@@ -49215,7 +49215,7 @@
         <v>8080</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>8330</v>
+        <v>1920</v>
       </c>
       <c r="K46" s="3" t="inlineStr"/>
       <c r="L46" s="3">
@@ -49258,7 +49258,7 @@
         <v>8080</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>8330</v>
+        <v>1707</v>
       </c>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2">
@@ -49301,7 +49301,7 @@
         <v>427500</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>441000</v>
+        <v>853333</v>
       </c>
       <c r="K48" s="3" t="inlineStr"/>
       <c r="L48" s="3">
@@ -49344,7 +49344,7 @@
         <v>266</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>274</v>
+        <v>390</v>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2">
@@ -49387,7 +49387,7 @@
         <v>266</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>274</v>
+        <v>1200</v>
       </c>
       <c r="K50" s="3" t="inlineStr"/>
       <c r="L50" s="3">
@@ -49473,7 +49473,7 @@
         <v>1140</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>1180</v>
+        <v>12700</v>
       </c>
       <c r="K52" s="3" t="inlineStr"/>
       <c r="L52" s="3">
@@ -49516,7 +49516,7 @@
         <v>266</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>274</v>
+        <v>1270</v>
       </c>
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2">
@@ -49559,7 +49559,7 @@
         <v>1140</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>1180</v>
+        <v>6</v>
       </c>
       <c r="K54" s="3" t="inlineStr"/>
       <c r="L54" s="3">
@@ -49602,7 +49602,7 @@
         <v>1140</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1180</v>
+        <v>6</v>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2">
@@ -50849,7 +50849,7 @@
         <v>304</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>314</v>
+        <v>600</v>
       </c>
       <c r="K84" s="3" t="inlineStr"/>
       <c r="L84" s="3">
@@ -51537,7 +51537,7 @@
         <v>810</v>
       </c>
       <c r="J100" s="3" t="n">
-        <v>830</v>
+        <v>2480</v>
       </c>
       <c r="K100" s="3" t="inlineStr"/>
       <c r="L100" s="3">
@@ -51881,7 +51881,7 @@
         <v>14250</v>
       </c>
       <c r="J108" s="3" t="n">
-        <v>14700</v>
+        <v>9390000</v>
       </c>
       <c r="K108" s="3" t="inlineStr"/>
       <c r="L108" s="3">
@@ -51924,7 +51924,7 @@
         <v>14250</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>14700</v>
+        <v>20020000</v>
       </c>
       <c r="K109" s="2" t="inlineStr"/>
       <c r="L109" s="2">
@@ -51967,7 +51967,7 @@
         <v>14250</v>
       </c>
       <c r="J110" s="3" t="n">
-        <v>14700</v>
+        <v>300000</v>
       </c>
       <c r="K110" s="3" t="inlineStr"/>
       <c r="L110" s="3">
@@ -52010,7 +52010,7 @@
         <v>14250</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>14700</v>
+        <v>5660000</v>
       </c>
       <c r="K111" s="2" t="inlineStr"/>
       <c r="L111" s="2">
@@ -52053,7 +52053,7 @@
         <v>14250</v>
       </c>
       <c r="J112" s="3" t="n">
-        <v>14700</v>
+        <v>4500000</v>
       </c>
       <c r="K112" s="3" t="inlineStr"/>
       <c r="L112" s="3">
@@ -52096,7 +52096,7 @@
         <v>427500</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>441000</v>
+        <v>11270000</v>
       </c>
       <c r="K113" s="2" t="inlineStr"/>
       <c r="L113" s="2">
@@ -52182,7 +52182,7 @@
         <v>427500</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>441000</v>
+        <v>34390000</v>
       </c>
       <c r="K115" s="2" t="inlineStr"/>
       <c r="L115" s="2">
@@ -52225,7 +52225,7 @@
         <v>427500</v>
       </c>
       <c r="J116" s="3" t="n">
-        <v>441000</v>
+        <v>9140000</v>
       </c>
       <c r="K116" s="3" t="inlineStr"/>
       <c r="L116" s="3">
@@ -52268,7 +52268,7 @@
         <v>427500</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>441000</v>
+        <v>27520000</v>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
       <c r="L117" s="2">
@@ -52612,7 +52612,7 @@
         <v>266</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>274</v>
+        <v>590</v>
       </c>
       <c r="K125" s="2" t="inlineStr"/>
       <c r="L125" s="2">
@@ -52784,7 +52784,7 @@
         <v>1140</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>1180</v>
+        <v>11</v>
       </c>
       <c r="K129" s="2" t="inlineStr"/>
       <c r="L129" s="2">
@@ -52827,7 +52827,7 @@
         <v>1140</v>
       </c>
       <c r="J130" s="3" t="n">
-        <v>1180</v>
+        <v>11</v>
       </c>
       <c r="K130" s="3" t="inlineStr"/>
       <c r="L130" s="3">
@@ -53429,7 +53429,7 @@
         <v>142</v>
       </c>
       <c r="J144" s="3" t="n">
-        <v>147</v>
+        <v>8</v>
       </c>
       <c r="K144" s="3" t="inlineStr"/>
       <c r="L144" s="3">
@@ -53472,7 +53472,7 @@
         <v>810</v>
       </c>
       <c r="J145" s="2" t="n">
-        <v>830</v>
+        <v>26240</v>
       </c>
       <c r="K145" s="2" t="inlineStr"/>
       <c r="L145" s="2">
@@ -53515,7 +53515,7 @@
         <v>810</v>
       </c>
       <c r="J146" s="3" t="n">
-        <v>830</v>
+        <v>1080</v>
       </c>
       <c r="K146" s="3" t="inlineStr"/>
       <c r="L146" s="3">
@@ -53558,7 +53558,7 @@
         <v>810</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>830</v>
+        <v>1080</v>
       </c>
       <c r="K147" s="2" t="inlineStr"/>
       <c r="L147" s="2">
@@ -54332,7 +54332,7 @@
         <v>209000</v>
       </c>
       <c r="J165" s="2" t="n">
-        <v>215600</v>
+        <v>390000</v>
       </c>
       <c r="K165" s="2" t="inlineStr"/>
       <c r="L165" s="2">

</xml_diff>